<commit_message>
feat: Add web security environment, generate vulnerability reports, and update evaluation form.
</commit_message>
<xml_diff>
--- a/Evaluation Form.xlsx
+++ b/Evaluation Form.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.109375" customWidth="1" min="1" max="1"/>
@@ -513,18 +513,18 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mass Assignment</t>
+          <t>SQL Injection</t>
         </is>
       </c>
       <c r="D2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -536,11 +536,11 @@
     <row r="3">
       <c r="C3" t="inlineStr">
         <is>
-          <t>SQL Injection</t>
+          <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -552,41 +552,41 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="C4" t="inlineStr">
         <is>
-          <t>IDOR</t>
+          <t>Insecure Direct Object Reference (IDOR)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="C5" t="inlineStr">
         <is>
-          <t>Broken Access Control</t>
+          <t>Broken Access Control (BAC)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -598,18 +598,18 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" t="inlineStr">
         <is>
-          <t>Negative Quantity</t>
+          <t>Cross-Site Request Forgery (CSRF)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -628,11 +628,11 @@
     <row r="7">
       <c r="C7" t="inlineStr">
         <is>
-          <t>Race Condition</t>
+          <t>Insecure Deserialization</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -644,18 +644,18 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="C8" t="inlineStr">
         <is>
-          <t>Client-Side Price Manipulation</t>
+          <t>Mass Assignment</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -667,18 +667,18 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="C9" t="inlineStr">
         <is>
-          <t>Payment Bypass</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -697,11 +697,11 @@
     <row r="10">
       <c r="C10" t="inlineStr">
         <is>
-          <t>Information Disclosure</t>
+          <t>Sensitive Data Exposure</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -713,26 +713,18 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Social Media (5003)</t>
-        </is>
-      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Weak Password Policy</t>
+          <t>JWT Bypass</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -751,11 +743,11 @@
     <row r="12">
       <c r="C12" t="inlineStr">
         <is>
-          <t>Session Fixation</t>
+          <t>SAML Bypass</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -772,13 +764,21 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Social Media (5003)</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Weak Password Reset Token</t>
+          <t>SQL Injection</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -790,64 +790,64 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="C14" t="inlineStr">
         <is>
-          <t>IDOR</t>
+          <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="C15" t="inlineStr">
         <is>
-          <t>Stored XSS</t>
+          <t>Insecure Direct Object Reference (IDOR)</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="C16" t="inlineStr">
         <is>
-          <t>Reflected XSS</t>
+          <t>Cross-Site Request Forgery (CSRF)</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -859,18 +859,18 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="C17" t="inlineStr">
         <is>
-          <t>Unrestricted File Upload</t>
+          <t>File Upload</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -912,7 +912,7 @@
     <row r="19">
       <c r="C19" t="inlineStr">
         <is>
-          <t>CSRF</t>
+          <t>Sensitive Data Exposure</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -928,18 +928,18 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="C20" t="inlineStr">
         <is>
-          <t>SQL Injection</t>
+          <t>Weak Password</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -951,26 +951,18 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
-        <v>3</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Banking (5004)</t>
-        </is>
-      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CSRF</t>
+          <t>Session Fixation</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -982,25 +974,25 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="C22" t="inlineStr">
         <is>
-          <t>IDOR</t>
+          <t>Weak Reset Token</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1010,53 +1002,37 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OAuth Bypass</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>9</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>JWT Bypass</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
         <v>4</v>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Blog (5005)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Stored XSS</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>5</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>File Share (5006)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Unrestricted File Upload</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>1</v>
-      </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
@@ -1067,53 +1043,353 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Banking (5004)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
           <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>IDOR</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="C26" t="inlineStr">
         <is>
+          <t>Cross-Site Scripting (XSS)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Insecure Direct Object Reference (IDOR)</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cross-Site Request Forgery (CSRF)</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>9</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Blog (5005)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>17%</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Cross-Site Scripting (XSS)</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>13</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Server-Side Request Forgery (SSRF)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>JWT Bypass</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>5</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>File Share (5006)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Cross-Site Scripting (XSS)</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Insecure Direct Object Reference (IDOR)</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>File Upload</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="C37" t="inlineStr">
+        <is>
           <t>Path Traversal</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Command Injection</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: focus autonomous scans on high-value actions and refresh evaluation
</commit_message>
<xml_diff>
--- a/Evaluation Form.xlsx
+++ b/Evaluation Form.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="7260" yWindow="3756" windowWidth="23040" windowHeight="12120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.109375" customWidth="1" min="1" max="1"/>
@@ -517,14 +517,14 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>67%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -540,14 +540,14 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -563,14 +563,14 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -586,14 +586,14 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -605,11 +605,11 @@
     <row r="6">
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cross-Site Request Forgery (CSRF)</t>
+          <t>Insecure Deserialization</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -621,18 +621,18 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="C7" t="inlineStr">
         <is>
-          <t>Insecure Deserialization</t>
+          <t>Mass Assignment</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -644,64 +644,64 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mass Assignment</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="C9" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Sensitive Data Exposure</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sensitive Data Exposure</t>
+          <t>JWT Bypass</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -718,43 +718,51 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Social Media (5003)</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>JWT Bypass</t>
+          <t>SQL Injection</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="C12" t="inlineStr">
         <is>
-          <t>SAML Bypass</t>
+          <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -764,21 +772,13 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Social Media (5003)</t>
-        </is>
-      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SQL Injection</t>
+          <t>Insecure Direct Object Reference (IDOR)</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -790,64 +790,64 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cross-Site Scripting (XSS)</t>
+          <t>Cross-Site Request Forgery (CSRF)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="C15" t="inlineStr">
         <is>
-          <t>Insecure Direct Object Reference (IDOR)</t>
+          <t>File Upload</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cross-Site Request Forgery (CSRF)</t>
+          <t>Path Traversal</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -859,18 +859,18 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="C17" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Weak Password</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -882,25 +882,25 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="C18" t="inlineStr">
         <is>
-          <t>Path Traversal</t>
+          <t>Session Fixation</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -912,18 +912,18 @@
     <row r="19">
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sensitive Data Exposure</t>
+          <t>Weak Reset Token</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -935,11 +935,11 @@
     <row r="20">
       <c r="C20" t="inlineStr">
         <is>
-          <t>Weak Password</t>
+          <t>OAuth Bypass</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -958,11 +958,11 @@
     <row r="21">
       <c r="C21" t="inlineStr">
         <is>
-          <t>Session Fixation</t>
+          <t>JWT Bypass</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -979,20 +979,28 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Banking (5004)</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Weak Reset Token</t>
+          <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1004,11 +1012,11 @@
     <row r="23">
       <c r="C23" t="inlineStr">
         <is>
-          <t>OAuth Bypass</t>
+          <t>Insecure Direct Object Reference (IDOR)</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1020,79 +1028,79 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="C24" t="inlineStr">
         <is>
-          <t>JWT Bypass</t>
+          <t>Cross-Site Request Forgery (CSRF)</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Banking (5004)</t>
+          <t>Blog (5005)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SQL Injection</t>
+          <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>4</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cross-Site Scripting (XSS)</t>
+          <t>Server-Side Request Forgery (SSRF)</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1104,88 +1112,88 @@
     <row r="27">
       <c r="C27" t="inlineStr">
         <is>
+          <t>JWT Bypass</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>File Share (5006)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cross-Site Scripting (XSS)</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" t="inlineStr">
+        <is>
           <t>Insecure Direct Object Reference (IDOR)</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>8</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
         <is>
           <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Cross-Site Request Forgery (CSRF)</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>9</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>4</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Blog (5005)</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>SQL Injection</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>6</v>
-      </c>
-      <c r="E29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>17%</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="C30" t="inlineStr">
         <is>
-          <t>Cross-Site Scripting (XSS)</t>
+          <t>File Upload</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
@@ -1197,18 +1205,18 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="C31" t="inlineStr">
         <is>
-          <t>Server-Side Request Forgery (SSRF)</t>
+          <t>Path Traversal</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
@@ -1227,167 +1235,21 @@
     <row r="32">
       <c r="C32" t="inlineStr">
         <is>
-          <t>JWT Bypass</t>
+          <t>Command Injection</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>5</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>File Share (5006)</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>SQL Injection</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>3</v>
-      </c>
-      <c r="E33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Cross-Site Scripting (XSS)</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>3</v>
-      </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Insecure Direct Object Reference (IDOR)</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>8</v>
-      </c>
-      <c r="E35" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>12%</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>File Upload</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>7</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Path Traversal</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>2</v>
-      </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Command Injection</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>5</v>
-      </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>

</xml_diff>